<commit_message>
data: EP1 extract → realistically-messy version (mixed encodings/sentinels/date formats; same patients)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EP1_cohort/cohort_extract.xlsx
+++ b/EP1_cohort/cohort_extract.xlsx
@@ -548,12 +548,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025/03/16</t>
+          <t>2025-03-16</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2025/03/24</t>
+          <t>03/24/2025</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -567,11 +567,15 @@
       <c r="J2" t="n">
         <v>0</v>
       </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>5.9</v>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5.9 </t>
+        </is>
       </c>
       <c r="M2" t="n">
         <v>11.3</v>
@@ -604,7 +608,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -612,12 +616,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/01/16</t>
+          <t>01/16/2025</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/01/31</t>
+          <t>01/31/2025</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -628,11 +632,18 @@
           <t>泌尿道感染</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>999</v>
       </c>
       <c r="M3" t="n">
         <v>10.5</v>
@@ -640,8 +651,10 @@
       <c r="N3" t="n">
         <v>2.47</v>
       </c>
-      <c r="O3" t="n">
-        <v>1</v>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -678,7 +691,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025/02/09</t>
+          <t>2025-02-09</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -686,14 +699,16 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>肺炎</t>
+          <t xml:space="preserve">肺炎 </t>
         </is>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" t="n">
-        <v>1</v>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L4" t="n">
         <v>12.8</v>
@@ -729,7 +744,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -737,7 +752,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2025/05/03</t>
+          <t>2025-05-03</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -753,8 +768,10 @@
           <t>腦中風</t>
         </is>
       </c>
-      <c r="J5" t="n">
-        <v>1</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="K5" t="n">
         <v>1</v>
@@ -768,8 +785,10 @@
       <c r="N5" t="n">
         <v>0.98</v>
       </c>
-      <c r="O5" t="n">
-        <v>0</v>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
@@ -801,7 +820,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025/02/28</t>
+          <t>2025-02-28</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -817,11 +836,15 @@
           <t>肺炎</t>
         </is>
       </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L6" t="n">
         <v>17.6</v>
@@ -865,12 +888,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2024/10/17</t>
+          <t>10/17/2024</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2024/10/19</t>
+          <t>2024-10-19</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -896,8 +919,10 @@
       <c r="N7" t="n">
         <v>1.69</v>
       </c>
-      <c r="O7" t="n">
-        <v>1</v>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -929,7 +954,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2024/06/04</t>
+          <t>06/04/2024</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -948,8 +973,13 @@
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>999</v>
       </c>
       <c r="M8" t="n">
         <v>11</v>
@@ -957,8 +987,10 @@
       <c r="N8" t="n">
         <v>1.21</v>
       </c>
-      <c r="O8" t="n">
-        <v>1</v>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q8" t="n">
         <v>1</v>
@@ -995,7 +1027,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2025/01/02</t>
+          <t>2025-01-02</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -1054,12 +1086,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2024/06/22</t>
+          <t>06/22/2024</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2024/07/02</t>
+          <t>2024-07-02</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -1085,8 +1117,10 @@
       <c r="N10" t="n">
         <v>0.76</v>
       </c>
-      <c r="O10" t="n">
-        <v>1</v>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1123,7 +1157,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2024/08/14</t>
+          <t>08/14/2024</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -1131,14 +1165,18 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>肺炎</t>
-        </is>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
+          <t xml:space="preserve">肺炎 </t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="L11" t="n">
         <v>9.800000000000001</v>
@@ -1174,7 +1212,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -1182,12 +1220,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2024/01/21</t>
+          <t>2024-01-21</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2024/01/25</t>
+          <t>2024-01-25</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -1201,8 +1239,10 @@
       <c r="J12" t="n">
         <v>1</v>
       </c>
-      <c r="K12" t="n">
-        <v>1</v>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L12" t="n">
         <v>7.7</v>
@@ -1213,8 +1253,10 @@
       <c r="N12" t="n">
         <v>0.54</v>
       </c>
-      <c r="O12" t="n">
-        <v>1</v>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -1251,7 +1293,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2024/01/31</t>
+          <t>01/31/2024</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -1310,12 +1352,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2024/10/09</t>
+          <t>2024-10-09</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2024/10/15</t>
+          <t>2024-10-15</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -1323,14 +1365,18 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>腦中風</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" t="n">
-        <v>1</v>
+          <t xml:space="preserve">腦中風 </t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L14" t="n">
         <v>4.9</v>
@@ -1366,7 +1412,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -1374,12 +1420,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2024/01/07</t>
+          <t>2024-01-07</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2024/01/15</t>
+          <t>01/15/2024</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -1405,8 +1451,10 @@
       <c r="N15" t="n">
         <v>1.62</v>
       </c>
-      <c r="O15" t="n">
-        <v>1</v>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -1443,7 +1491,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2025/02/06</t>
+          <t>2025-02-06</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -1454,8 +1502,10 @@
           <t>蜂窩性組織炎</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>0</v>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1502,7 +1552,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2024/01/10</t>
+          <t>01/10/2024</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1518,11 +1568,15 @@
           <t>泌尿道感染</t>
         </is>
       </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>1</v>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L17" t="n">
         <v>15.6</v>
@@ -1558,7 +1612,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E18" t="n">
@@ -1571,7 +1625,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2024/11/03</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -1579,7 +1633,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>糖尿病酮酸中毒</t>
+          <t xml:space="preserve">糖尿病酮酸中毒 </t>
         </is>
       </c>
       <c r="J18" t="n">
@@ -1630,7 +1684,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2024/08/06</t>
+          <t>08/06/2024</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1646,11 +1700,15 @@
           <t>腦中風</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>1</v>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L19" t="n">
         <v>8.300000000000001</v>
@@ -1686,7 +1744,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -1694,7 +1752,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2025/06/24</t>
+          <t>2025-06-24</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1710,14 +1768,20 @@
           <t>蜂窩性組織炎</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>4.2</v>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 4.2 </t>
+        </is>
       </c>
       <c r="M20" t="n">
         <v>10.2</v>
@@ -1758,7 +1822,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2024/12/25</t>
+          <t>2024-12-25</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1777,8 +1841,10 @@
       <c r="J21" t="n">
         <v>0</v>
       </c>
-      <c r="K21" t="n">
-        <v>0</v>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="L21" t="n">
         <v>13.2</v>
@@ -1822,12 +1888,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2024/04/20</t>
+          <t>2024-04-20</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2024/04/27</t>
+          <t>04/27/2024</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -1844,6 +1910,9 @@
       <c r="K22" t="n">
         <v>1</v>
       </c>
+      <c r="L22" t="n">
+        <v>999</v>
+      </c>
       <c r="M22" t="n">
         <v>12.9</v>
       </c>
@@ -1883,12 +1952,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2024/11/08</t>
+          <t>2024-11-08</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2024/11/13</t>
+          <t>2024-11-13</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -1911,11 +1980,15 @@
       <c r="M23" t="n">
         <v>14.9</v>
       </c>
-      <c r="N23" t="n">
-        <v>3.15</v>
-      </c>
-      <c r="O23" t="n">
-        <v>0</v>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>未測</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -1939,7 +2012,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1947,12 +2020,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2025/02/08</t>
+          <t>02/08/2025</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2025/02/12</t>
+          <t>02/12/2025</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -1963,8 +2036,10 @@
           <t>泌尿道感染</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>1</v>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -2011,12 +2086,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2025/01/09</t>
+          <t>01/09/2025</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2025/01/20</t>
+          <t>2025-01-20</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -2027,11 +2102,15 @@
           <t>糖尿病酮酸中毒</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>1</v>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L25" t="n">
         <v>2.8</v>
@@ -2042,8 +2121,10 @@
       <c r="N25" t="n">
         <v>1.84</v>
       </c>
-      <c r="O25" t="n">
-        <v>0</v>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="Q25" t="n">
         <v>1</v>
@@ -2075,7 +2156,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2024/01/02</t>
+          <t>01/02/2024</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2088,11 +2169,13 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>心衰竭</t>
-        </is>
-      </c>
-      <c r="J26" t="n">
-        <v>0</v>
+          <t xml:space="preserve">心衰竭 </t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -2100,6 +2183,9 @@
       <c r="L26" t="n">
         <v>5.4</v>
       </c>
+      <c r="M26" t="n">
+        <v>999</v>
+      </c>
       <c r="N26" t="n">
         <v>1.48</v>
       </c>
@@ -2128,7 +2214,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -2136,12 +2222,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2024/10/10</t>
+          <t>2024-10-10</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2024/10/15</t>
+          <t>10/15/2024</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -2155,8 +2241,15 @@
       <c r="J27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="n">
-        <v>1</v>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>未檢</t>
+        </is>
       </c>
       <c r="M27" t="n">
         <v>9.6</v>
@@ -2197,7 +2290,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2024/01/13</t>
+          <t>2024-01-13</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2213,8 +2306,10 @@
           <t>蜂窩性組織炎</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>1</v>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -2228,8 +2323,10 @@
       <c r="N28" t="n">
         <v>1.94</v>
       </c>
-      <c r="O28" t="n">
-        <v>1</v>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q28" t="n">
         <v>1</v>
@@ -2266,7 +2363,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2025/06/25</t>
+          <t>06/25/2025</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -2280,11 +2377,15 @@
       <c r="J29" t="n">
         <v>0</v>
       </c>
-      <c r="K29" t="n">
-        <v>1</v>
-      </c>
-      <c r="L29" t="n">
-        <v>4.8</v>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 4.8 </t>
+        </is>
       </c>
       <c r="M29" t="n">
         <v>12.7</v>
@@ -2344,8 +2445,10 @@
       <c r="J30" t="n">
         <v>1</v>
       </c>
-      <c r="K30" t="n">
-        <v>1</v>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L30" t="n">
         <v>10.7</v>
@@ -2381,7 +2484,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2394,7 +2497,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2024/06/11</t>
+          <t>06/11/2024</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -2405,11 +2508,20 @@
           <t>肺炎</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" t="n">
-        <v>1</v>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>未檢</t>
+        </is>
       </c>
       <c r="M31" t="n">
         <v>11</v>
@@ -2417,8 +2529,10 @@
       <c r="N31" t="n">
         <v>2.19</v>
       </c>
-      <c r="O31" t="n">
-        <v>1</v>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q31" t="n">
         <v>0</v>
@@ -2455,7 +2569,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2024/08/27</t>
+          <t>08/27/2024</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -2481,8 +2595,10 @@
       <c r="N32" t="n">
         <v>0.53</v>
       </c>
-      <c r="O32" t="n">
-        <v>1</v>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q32" t="n">
         <v>0</v>
@@ -2519,7 +2635,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2025/02/27</t>
+          <t>2025-02-27</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -2533,8 +2649,10 @@
       <c r="J33" t="n">
         <v>1</v>
       </c>
-      <c r="K33" t="n">
-        <v>1</v>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L33" t="n">
         <v>4</v>
@@ -2545,8 +2663,10 @@
       <c r="N33" t="n">
         <v>2.29</v>
       </c>
-      <c r="O33" t="n">
-        <v>0</v>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="Q33" t="n">
         <v>0</v>
@@ -2591,11 +2711,13 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>腦中風</t>
-        </is>
-      </c>
-      <c r="J34" t="n">
-        <v>0</v>
+          <t xml:space="preserve">腦中風 </t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -2603,8 +2725,13 @@
       <c r="L34" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="N34" t="n">
-        <v>1.46</v>
+      <c r="M34" t="n">
+        <v>999</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>未測</t>
+        </is>
       </c>
       <c r="O34" t="n">
         <v>0</v>
@@ -2631,7 +2758,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2639,7 +2766,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2024/11/13</t>
+          <t>11/13/2024</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2655,8 +2782,10 @@
           <t>糖尿病酮酸中毒</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>1</v>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="K35" t="n">
         <v>1</v>
@@ -2670,8 +2799,10 @@
       <c r="N35" t="n">
         <v>1.05</v>
       </c>
-      <c r="O35" t="n">
-        <v>1</v>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q35" t="n">
         <v>0</v>
@@ -2695,7 +2826,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -2703,12 +2834,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2024/05/28</t>
+          <t>05/28/2024</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2024/05/29</t>
+          <t>05/29/2024</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -2772,7 +2903,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2024/01/19</t>
+          <t>2024-01-19</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -2786,8 +2917,10 @@
       <c r="J37" t="n">
         <v>1</v>
       </c>
-      <c r="K37" t="n">
-        <v>1</v>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L37" t="n">
         <v>6.8</v>
@@ -2798,8 +2931,10 @@
       <c r="N37" t="n">
         <v>2.65</v>
       </c>
-      <c r="O37" t="n">
-        <v>0</v>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="Q37" t="n">
         <v>0</v>
@@ -2823,7 +2958,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2836,7 +2971,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2025/03/19</t>
+          <t>03/19/2025</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -2862,8 +2997,10 @@
       <c r="N38" t="n">
         <v>2.61</v>
       </c>
-      <c r="O38" t="n">
-        <v>1</v>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q38" t="n">
         <v>0</v>
@@ -2895,12 +3032,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2025/01/26</t>
+          <t>01/26/2025</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2025/02/01</t>
+          <t>2025-02-01</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -2914,8 +3051,10 @@
       <c r="J39" t="n">
         <v>0</v>
       </c>
-      <c r="K39" t="n">
-        <v>1</v>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L39" t="n">
         <v>9.6</v>
@@ -2964,7 +3103,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2024/04/28</t>
+          <t>04/28/2024</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -2975,14 +3114,20 @@
           <t>腦中風</t>
         </is>
       </c>
-      <c r="J40" t="n">
-        <v>0</v>
-      </c>
-      <c r="K40" t="n">
-        <v>1</v>
-      </c>
-      <c r="L40" t="n">
-        <v>12.8</v>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 12.8 </t>
+        </is>
       </c>
       <c r="M40" t="n">
         <v>13</v>
@@ -2990,8 +3135,10 @@
       <c r="N40" t="n">
         <v>2.29</v>
       </c>
-      <c r="O40" t="n">
-        <v>1</v>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q40" t="n">
         <v>0</v>
@@ -3023,12 +3170,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2025/03/06</t>
+          <t>2025-03-06</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2025/03/12</t>
+          <t>03/12/2025</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -3036,11 +3183,13 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>腦中風</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
-        <v>0</v>
+          <t xml:space="preserve">腦中風 </t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="K41" t="n">
         <v>1</v>
@@ -3048,6 +3197,9 @@
       <c r="L41" t="n">
         <v>14.2</v>
       </c>
+      <c r="M41" t="n">
+        <v>999</v>
+      </c>
       <c r="N41" t="n">
         <v>2.06</v>
       </c>
@@ -3084,12 +3236,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2025/03/11</t>
+          <t>2025-03-11</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2025/03/15</t>
+          <t>2025-03-15</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -3100,11 +3252,15 @@
           <t>急性腎損傷</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K42" t="n">
-        <v>1</v>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L42" t="n">
         <v>11.9</v>
@@ -3148,12 +3304,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2024/03/03</t>
+          <t>03/03/2024</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2024/03/08</t>
+          <t>03/08/2024</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -3164,8 +3320,10 @@
           <t>泌尿道感染</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>1</v>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="K43" t="n">
         <v>1</v>
@@ -3176,8 +3334,10 @@
       <c r="M43" t="n">
         <v>10.6</v>
       </c>
-      <c r="N43" t="n">
-        <v>0.89</v>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>未測</t>
+        </is>
       </c>
       <c r="O43" t="n">
         <v>0</v>
@@ -3212,12 +3372,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2024/07/31</t>
+          <t>07/31/2024</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2024/08/04</t>
+          <t>2024-08-04</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -3228,11 +3388,15 @@
           <t>泌尿道感染</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>1</v>
-      </c>
-      <c r="K44" t="n">
-        <v>1</v>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L44" t="n">
         <v>3.7</v>
@@ -3243,8 +3407,10 @@
       <c r="N44" t="n">
         <v>1.58</v>
       </c>
-      <c r="O44" t="n">
-        <v>1</v>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="P44" t="n">
         <v>1</v>
@@ -3271,7 +3437,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -3279,12 +3445,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2024/11/06</t>
+          <t>2024-11-06</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2024/11/10</t>
+          <t>11/10/2024</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -3295,8 +3461,10 @@
           <t>泌尿道感染</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>1</v>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="K45" t="n">
         <v>1</v>
@@ -3307,11 +3475,15 @@
       <c r="M45" t="n">
         <v>11.4</v>
       </c>
-      <c r="N45" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="O45" t="n">
-        <v>1</v>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>未測</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="P45" t="n">
         <v>1</v>
@@ -3346,12 +3518,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2024/08/25</t>
+          <t>2024-08-25</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2024/09/07</t>
+          <t>2024-09-07</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -3362,11 +3534,15 @@
           <t>糖尿病酮酸中毒</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>0</v>
-      </c>
-      <c r="K46" t="n">
-        <v>0</v>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="L46" t="n">
         <v>6.2</v>
@@ -3415,7 +3591,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2024/01/19</t>
+          <t>2024-01-19</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -3423,17 +3599,24 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>糖尿病酮酸中毒</t>
-        </is>
-      </c>
-      <c r="J47" t="n">
-        <v>0</v>
+          <t xml:space="preserve">糖尿病酮酸中毒 </t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
       </c>
       <c r="K47" t="n">
         <v>1</v>
       </c>
-      <c r="L47" t="n">
-        <v>10.6</v>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 10.6 </t>
+        </is>
+      </c>
+      <c r="M47" t="n">
+        <v>999</v>
       </c>
       <c r="N47" t="n">
         <v>2.81</v>
@@ -3476,7 +3659,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2024/06/29</t>
+          <t>06/29/2024</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -3487,11 +3670,15 @@
           <t>心衰竭</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>1</v>
-      </c>
-      <c r="K48" t="n">
-        <v>1</v>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="L48" t="n">
         <v>4.5</v>
@@ -3540,7 +3727,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2024/07/15</t>
+          <t>07/15/2024</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -3566,8 +3753,10 @@
       <c r="N49" t="n">
         <v>1.2</v>
       </c>
-      <c r="O49" t="n">
-        <v>1</v>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
       </c>
       <c r="Q49" t="n">
         <v>0</v>

</xml_diff>